<commit_message>
Data to 22 October; sheet for 22-28 October
Results and referee appointments collected by the daily job since 15 October,
and the first automatically built sheet: Walsall v Salford, 26 October.
</commit_message>
<xml_diff>
--- a/forward_test_2026-09-18.xlsx
+++ b/forward_test_2026-09-18.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Week 26 Sep" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Week 9-12 Oct" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Week 3 Oct" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Week 22-28 Oct" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -189,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -290,6 +291,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12553,7 +12560,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="35" t="inlineStr">
         <is>
@@ -12616,8 +12622,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="48" t="inlineStr">
         <is>
@@ -24405,4 +24409,722 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:BD35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+    <col width="7" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="22" max="22"/>
+    <col width="8" customWidth="1" min="23" max="23"/>
+    <col width="8" customWidth="1" min="24" max="24"/>
+    <col width="8" customWidth="1" min="25" max="25"/>
+    <col width="8" customWidth="1" min="26" max="26"/>
+    <col width="8" customWidth="1" min="27" max="27"/>
+    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
+    <col width="13" customWidth="1" min="35" max="35"/>
+    <col width="13" customWidth="1" min="36" max="36"/>
+    <col width="13" customWidth="1" min="37" max="37"/>
+    <col width="13" customWidth="1" min="38" max="38"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="13" customWidth="1" min="41" max="41"/>
+    <col width="17" customWidth="1" min="42" max="42"/>
+    <col width="9" customWidth="1" min="43" max="43"/>
+    <col width="10" customWidth="1" min="44" max="44"/>
+    <col width="11" customWidth="1" min="45" max="45"/>
+    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="13" customWidth="1" min="47" max="47"/>
+    <col width="14" customWidth="1" min="48" max="48"/>
+    <col width="8" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="9" customWidth="1" min="51" max="51"/>
+    <col width="14" customWidth="1" min="52" max="52"/>
+    <col width="8" customWidth="1" min="53" max="53"/>
+    <col width="9" customWidth="1" min="54" max="54"/>
+    <col width="12" customWidth="1" min="55" max="55"/>
+    <col width="34" customWidth="1" min="56" max="56"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="24" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="24" t="inlineStr">
+        <is>
+          <t>Div</t>
+        </is>
+      </c>
+      <c r="C1" s="24" t="inlineStr">
+        <is>
+          <t>League</t>
+        </is>
+      </c>
+      <c r="D1" s="24" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="E1" s="24" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>Referee</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>Ref matches</t>
+        </is>
+      </c>
+      <c r="H1" s="24" t="inlineStr">
+        <is>
+          <t>Ref vs avg</t>
+        </is>
+      </c>
+      <c r="I1" s="24" t="inlineStr">
+        <is>
+          <t>League avg</t>
+        </is>
+      </c>
+      <c r="J1" s="24" t="inlineStr">
+        <is>
+          <t>Model expects</t>
+        </is>
+      </c>
+      <c r="K1" s="24" t="inlineStr">
+        <is>
+          <t>vs league avg</t>
+        </is>
+      </c>
+      <c r="L1" s="24" t="inlineStr">
+        <is>
+          <t>Most likely</t>
+        </is>
+      </c>
+      <c r="M1" s="24" t="inlineStr">
+        <is>
+          <t>80% range</t>
+        </is>
+      </c>
+      <c r="N1" s="24" t="inlineStr">
+        <is>
+          <t>P(0)</t>
+        </is>
+      </c>
+      <c r="O1" s="24" t="inlineStr">
+        <is>
+          <t>P(1)</t>
+        </is>
+      </c>
+      <c r="P1" s="24" t="inlineStr">
+        <is>
+          <t>P(2)</t>
+        </is>
+      </c>
+      <c r="Q1" s="24" t="inlineStr">
+        <is>
+          <t>P(3)</t>
+        </is>
+      </c>
+      <c r="R1" s="24" t="inlineStr">
+        <is>
+          <t>P(4)</t>
+        </is>
+      </c>
+      <c r="S1" s="24" t="inlineStr">
+        <is>
+          <t>P(5)</t>
+        </is>
+      </c>
+      <c r="T1" s="24" t="inlineStr">
+        <is>
+          <t>P(6)</t>
+        </is>
+      </c>
+      <c r="U1" s="24" t="inlineStr">
+        <is>
+          <t>P(7)</t>
+        </is>
+      </c>
+      <c r="V1" s="24" t="inlineStr">
+        <is>
+          <t>P(8)</t>
+        </is>
+      </c>
+      <c r="W1" s="24" t="inlineStr">
+        <is>
+          <t>P(o1.5)</t>
+        </is>
+      </c>
+      <c r="X1" s="24" t="inlineStr">
+        <is>
+          <t>P(o2.5)</t>
+        </is>
+      </c>
+      <c r="Y1" s="24" t="inlineStr">
+        <is>
+          <t>P(o3.5)</t>
+        </is>
+      </c>
+      <c r="Z1" s="24" t="inlineStr">
+        <is>
+          <t>P(o4.5)</t>
+        </is>
+      </c>
+      <c r="AA1" s="24" t="inlineStr">
+        <is>
+          <t>P(o5.5)</t>
+        </is>
+      </c>
+      <c r="AB1" s="24" t="inlineStr">
+        <is>
+          <t>P(o6.5)</t>
+        </is>
+      </c>
+      <c r="AC1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR over 1.5</t>
+        </is>
+      </c>
+      <c r="AD1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR over 2.5</t>
+        </is>
+      </c>
+      <c r="AE1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR over 3.5</t>
+        </is>
+      </c>
+      <c r="AF1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR over 4.5</t>
+        </is>
+      </c>
+      <c r="AG1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR over 5.5</t>
+        </is>
+      </c>
+      <c r="AH1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR over 6.5</t>
+        </is>
+      </c>
+      <c r="AI1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR under 1.5</t>
+        </is>
+      </c>
+      <c r="AJ1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR under 2.5</t>
+        </is>
+      </c>
+      <c r="AK1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR under 3.5</t>
+        </is>
+      </c>
+      <c r="AL1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR under 4.5</t>
+        </is>
+      </c>
+      <c r="AM1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR under 5.5</t>
+        </is>
+      </c>
+      <c r="AN1" s="24" t="inlineStr">
+        <is>
+          <t>FAIR under 6.5</t>
+        </is>
+      </c>
+      <c r="AO1" s="25" t="inlineStr">
+        <is>
+          <t>Bookmaker</t>
+        </is>
+      </c>
+      <c r="AP1" s="25" t="inlineStr">
+        <is>
+          <t>Settles on</t>
+        </is>
+      </c>
+      <c r="AQ1" s="25" t="inlineStr">
+        <is>
+          <t>Card line</t>
+        </is>
+      </c>
+      <c r="AR1" s="25" t="inlineStr">
+        <is>
+          <t>Over price</t>
+        </is>
+      </c>
+      <c r="AS1" s="25" t="inlineStr">
+        <is>
+          <t>Under price</t>
+        </is>
+      </c>
+      <c r="AT1" s="25" t="inlineStr">
+        <is>
+          <t>Stake EUR</t>
+        </is>
+      </c>
+      <c r="AU1" s="24" t="inlineStr">
+        <is>
+          <t>Model P(over)</t>
+        </is>
+      </c>
+      <c r="AV1" s="24" t="inlineStr">
+        <is>
+          <t>Implied P(over)</t>
+        </is>
+      </c>
+      <c r="AW1" s="24" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="AX1" s="24" t="inlineStr">
+        <is>
+          <t>BET?</t>
+        </is>
+      </c>
+      <c r="AY1" s="24" t="inlineStr">
+        <is>
+          <t>EV EUR</t>
+        </is>
+      </c>
+      <c r="AZ1" s="25" t="inlineStr">
+        <is>
+          <t>ACTUAL yellows</t>
+        </is>
+      </c>
+      <c r="BA1" s="24" t="inlineStr">
+        <is>
+          <t>Won?</t>
+        </is>
+      </c>
+      <c r="BB1" s="24" t="inlineStr">
+        <is>
+          <t>P/L EUR</t>
+        </is>
+      </c>
+      <c r="BC1" s="24" t="inlineStr">
+        <is>
+          <t>Running P/L</t>
+        </is>
+      </c>
+      <c r="BD1" s="25" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="B2" s="26" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="C2" s="26" t="inlineStr">
+        <is>
+          <t>League Two</t>
+        </is>
+      </c>
+      <c r="D2" s="26" t="inlineStr">
+        <is>
+          <t>Walsall</t>
+        </is>
+      </c>
+      <c r="E2" s="26" t="inlineStr">
+        <is>
+          <t>Salford</t>
+        </is>
+      </c>
+      <c r="F2" s="27" t="inlineStr">
+        <is>
+          <t>m coy</t>
+        </is>
+      </c>
+      <c r="G2" s="26" t="n">
+        <v>213</v>
+      </c>
+      <c r="H2" s="28" t="n">
+        <v>-0.4490018148820326</v>
+      </c>
+      <c r="I2" s="29" t="n">
+        <v>3.992753623188406</v>
+      </c>
+      <c r="J2" s="29" t="n">
+        <v>3.295274393631539</v>
+      </c>
+      <c r="K2" s="30" t="n">
+        <v>-0.174686268019687</v>
+      </c>
+      <c r="L2" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="M2" s="26" t="inlineStr">
+        <is>
+          <t>1-5</t>
+        </is>
+      </c>
+      <c r="N2" s="31" t="n">
+        <v>0.04127989534019522</v>
+      </c>
+      <c r="O2" s="31" t="n">
+        <v>0.1273131546529031</v>
+      </c>
+      <c r="P2" s="31" t="n">
+        <v>0.2004045838105295</v>
+      </c>
+      <c r="Q2" s="31" t="n">
+        <v>0.2145855754175058</v>
+      </c>
+      <c r="R2" s="31" t="n">
+        <v>0.1757646842689452</v>
+      </c>
+      <c r="S2" s="31" t="n">
+        <v>0.1174258038543715</v>
+      </c>
+      <c r="T2" s="31" t="n">
+        <v>0.0666293017985575</v>
+      </c>
+      <c r="U2" s="31" t="n">
+        <v>0.03301546323174859</v>
+      </c>
+      <c r="V2" s="31" t="n">
+        <v>0.01457896098207048</v>
+      </c>
+      <c r="W2" s="28" t="n">
+        <v>0.8314069500069017</v>
+      </c>
+      <c r="X2" s="28" t="n">
+        <v>0.6310023661963722</v>
+      </c>
+      <c r="Y2" s="28" t="n">
+        <v>0.4164167907788664</v>
+      </c>
+      <c r="Z2" s="28" t="n">
+        <v>0.2406521065099212</v>
+      </c>
+      <c r="AA2" s="28" t="n">
+        <v>0.1232263026555497</v>
+      </c>
+      <c r="AB2" s="28" t="n">
+        <v>0.05659700085699215</v>
+      </c>
+      <c r="AC2" s="29" t="n">
+        <v>1.202780419374289</v>
+      </c>
+      <c r="AD2" s="29" t="n">
+        <v>1.584780111091997</v>
+      </c>
+      <c r="AE2" s="29" t="n">
+        <v>2.401440148774018</v>
+      </c>
+      <c r="AF2" s="29" t="n">
+        <v>4.15537605094171</v>
+      </c>
+      <c r="AG2" s="29" t="n">
+        <v>8.115150568099622</v>
+      </c>
+      <c r="AH2" s="29" t="n">
+        <v>17.66878076325589</v>
+      </c>
+      <c r="AI2" s="29" t="n">
+        <v>5.931442607159292</v>
+      </c>
+      <c r="AJ2" s="29" t="n">
+        <v>2.710044478312772</v>
+      </c>
+      <c r="AK2" s="29" t="n">
+        <v>1.713551699567621</v>
+      </c>
+      <c r="AL2" s="29" t="n">
+        <v>1.316919436496818</v>
+      </c>
+      <c r="AM2" s="29" t="n">
+        <v>1.140545163511148</v>
+      </c>
+      <c r="AN2" s="29" t="n">
+        <v>1.059992390217548</v>
+      </c>
+      <c r="AO2" s="27" t="n"/>
+      <c r="AP2" s="27" t="n"/>
+      <c r="AQ2" s="27" t="n"/>
+      <c r="AR2" s="27" t="n"/>
+      <c r="AS2" s="27" t="n"/>
+      <c r="AT2" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="AU2" s="32">
+        <f>IFERROR(IF($AQ2="","",INDEX($W2:$AB2,$AQ2-0.5)),"")</f>
+        <v/>
+      </c>
+      <c r="AV2" s="32">
+        <f>IF($AR2="","",IF($AS2="",1/$AR2,(1/$AR2)/((1/$AR2)+(1/$AS2))))</f>
+        <v/>
+      </c>
+      <c r="AW2" s="32">
+        <f>IF(OR($AU2="",$AV2=""),"",$AU2-$AV2)</f>
+        <v/>
+      </c>
+      <c r="AX2" s="33">
+        <f>IF($AW2="","",IF($AP2="","units?",IF(ISNUMBER(SEARCH("yellow",$AP2)),IF($AW2&gt;=0.05,"OVER",IF($AW2&lt;=-0.05,"UNDER","skip")),"UNITS?")))</f>
+        <v/>
+      </c>
+      <c r="AY2" s="34">
+        <f>IF(OR($AX2="",$AX2="skip",$AX2="units?",$AX2="UNITS?"),"",IF($AX2="OVER",$AT2*($AU2*$AR2-1),$AT2*((1-$AU2)*$AS2-1)))</f>
+        <v/>
+      </c>
+      <c r="AZ2" s="27" t="n"/>
+      <c r="BA2" s="33">
+        <f>IF(OR($AX2="",$AX2="skip",$AX2="units?",$AX2="UNITS?",$AZ2="",$AQ2=""),"",IF($AX2="OVER",IF($AZ2&gt;$AQ2,"WON","LOST"),IF($AZ2&lt;$AQ2,"WON","LOST")))</f>
+        <v/>
+      </c>
+      <c r="BB2" s="34">
+        <f>IF($BA2="","",IF($BA2="WON",IF($AX2="OVER",$AT2*($AR2-1),$AT2*($AS2-1)),-$AT2))</f>
+        <v/>
+      </c>
+      <c r="BC2" s="34">
+        <f>IF(COUNT($BB$2:$BB2)=0,"",SUM($BB$2:$BB2))</f>
+        <v/>
+      </c>
+      <c r="BD2" s="27" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>bets placed</t>
+        </is>
+      </c>
+      <c r="E5" s="37">
+        <f>COUNTIF($AX$2:$AX2,"OVER")+COUNTIF($AX$2:$AX2,"UNDER")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>bets won</t>
+        </is>
+      </c>
+      <c r="E6" s="37">
+        <f>COUNTIF($BA$2:$BA2,"WON")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>total staked</t>
+        </is>
+      </c>
+      <c r="E7" s="38">
+        <f>SUMPRODUCT(($BA$2:$BA2&lt;&gt;"")*$AT$2:$AT2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>profit / loss EUR</t>
+        </is>
+      </c>
+      <c r="E8" s="38">
+        <f>IF(COUNT($BB$2:$BB2)=0,"",SUM($BB$2:$BB2))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="36" t="inlineStr">
+        <is>
+          <t>return on stake</t>
+        </is>
+      </c>
+      <c r="E9" s="39">
+        <f>IF($E7=0,"",$E8/$E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="52" t="inlineStr">
+        <is>
+          <t>HOW TO USE THIS SHEET</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="53" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="53" t="inlineStr">
+        <is>
+          <t>1. Fill the yellow columns only. Everything green is computed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="53" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="53" t="inlineStr">
+        <is>
+          <t>2. 'Settles on' must say what the market actually pays out on. Write 'yellow cards' only if the bookmaker settles on yellows alone. If it says total cards or booking points, BET? shows UNITS? and gives no verdict -- on purpose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="53" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The model predicts yellows. Counting a red as two cards adds about 5-6 percentage points at every line, always upward, which is larger than the 5% edge threshold. Priced against the wrong market the model shows an OVER edge on nearly every game, and that looks identical to finding an edge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="53" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The market to look for is 'Yellow Cards', as in the Chelsea screenshot -- not 'Cards' and not 'Booking Points'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="53" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="53" t="inlineStr">
+        <is>
+          <t>3. Record BOTH sides of the price. With one side only, the de-vig cannot run and the implied probability is overstated by the whole margin, which invents edge that is not there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="53" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="53" t="inlineStr">
+        <is>
+          <t>4. Record the price when you see it, before kick-off. A price looked up afterwards is not one you could have taken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="53" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="53" t="inlineStr">
+        <is>
+          <t>5. Stake is EUR 100 a bet. Change the column if you want; the P/L follows it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="53" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="52" t="inlineStr">
+        <is>
+          <t>WHAT THIS SHEET IS AND IS NOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="53" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="53" t="inlineStr">
+        <is>
+          <t>1 fixtures. A sample this size tells you nothing about whether the model beats a bookmaker -- a verdict on profitability needs thousands of bets. Treat a single week as practice for the workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="53" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="53" t="inlineStr">
+        <is>
+          <t>The referee is 48% of the model's value. If the Referee column says 'not known', the EFL has not published appointments yet (they come one to three days ahead) and these are the weaker version of the model. Re-run run_week_sheet.py for the same dates once they are out and every unplayed row updates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="53" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="53" t="inlineStr">
+        <is>
+          <t>Model fingerprint d30beac40c73a847, frozen for the season.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="53" t="inlineStr">
+        <is>
+          <t>Scoring these results against the model is a holdout look.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Workbook as rewritten by the 15:30 scheduled run
The job's week-sheet step rebuilt 'Week 22-28 Oct' at 15:30 on 26 October. No cell, formula or stored value differs from the previous commit; only the file's internal bytes changed.
</commit_message>
<xml_diff>
--- a/forward_test_2026-09-18.xlsx
+++ b/forward_test_2026-09-18.xlsx
@@ -190,7 +190,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -291,6 +291,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
@@ -12623,134 +12629,134 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="48" t="inlineStr">
+      <c r="A25" s="52" t="inlineStr">
         <is>
           <t>HOW TO USE THIS SHEET</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="49" t="inlineStr"/>
+      <c r="A26" s="53" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="49" t="inlineStr">
+      <c r="A27" s="53" t="inlineStr">
         <is>
           <t>1. Fill the yellow columns only. Everything green is computed.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="49" t="inlineStr"/>
+      <c r="A28" s="53" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="49" t="inlineStr">
+      <c r="A29" s="53" t="inlineStr">
         <is>
           <t>2. 'Settles on' must say what the market actually pays out on. Write 'yellow cards' only if the bookmaker settles on yellows alone. If it says total cards or booking points, BET? shows UNITS? and gives no verdict -- on purpose.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="49" t="inlineStr"/>
+      <c r="A30" s="53" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="49" t="inlineStr">
+      <c r="A31" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">   The model predicts yellows. Counting a red as two cards adds about 5-6 percentage points at every line, always upward, which is larger than the 5% edge threshold. Priced against the wrong market the model shows an OVER edge on nearly every game, and that looks identical to finding an edge.</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="49" t="inlineStr"/>
+      <c r="A32" s="53" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="49" t="inlineStr">
+      <c r="A33" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">   The market to look for is 'Yellow Cards', as in the Chelsea screenshot -- not 'Cards' and not 'Booking Points'.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="49" t="inlineStr"/>
+      <c r="A34" s="53" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="49" t="inlineStr">
+      <c r="A35" s="53" t="inlineStr">
         <is>
           <t>3. Record BOTH sides of the price. With one side only, the de-vig cannot run and the implied probability is overstated by the whole margin, which invents edge that is not there.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="49" t="inlineStr"/>
+      <c r="A36" s="53" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="49" t="inlineStr">
+      <c r="A37" s="53" t="inlineStr">
         <is>
           <t>4. Record the price when you see it, before kick-off. A price looked up afterwards is not one you could have taken.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="49" t="inlineStr"/>
+      <c r="A38" s="53" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="49" t="inlineStr">
+      <c r="A39" s="53" t="inlineStr">
         <is>
           <t>5. Stake is EUR 100 a bet. Change the column if you want; the P/L follows it.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="49" t="inlineStr"/>
+      <c r="A40" s="53" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="48" t="inlineStr">
+      <c r="A41" s="52" t="inlineStr">
         <is>
           <t>WHAT THIS WEEK IS AND IS NOT</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="49" t="inlineStr"/>
+      <c r="A42" s="53" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="49" t="inlineStr">
+      <c r="A43" s="53" t="inlineStr">
         <is>
           <t>Fourteen fixtures, League One and League Two only -- 26 September starts a two-weekend international break, and seven more EFL matches are postponed. No Premier League or Championship football until 10 October.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="49" t="inlineStr"/>
+      <c r="A44" s="53" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="49" t="inlineStr">
+      <c r="A45" s="53" t="inlineStr">
         <is>
           <t>Fourteen matches is far too few to tell you anything about whether the model beats a bookmaker. Treat this as practice for the workflow. A verdict on profitability needs thousands of bets.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="49" t="inlineStr"/>
+      <c r="A46" s="53" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="49" t="inlineStr">
+      <c r="A47" s="53" t="inlineStr">
         <is>
           <t>Referees are not in yet. The EFL publishes appointments one to three days ahead, and the referee is 48% of the model's value -- so these numbers are the weaker version of the model. Re-run cards/run_week_sheet.py once the appointments are out.</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="49" t="inlineStr"/>
+      <c r="A48" s="53" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="49" t="inlineStr">
+      <c r="A49" s="53" t="inlineStr">
         <is>
           <t>Model fingerprint d30beac40c73a847, frozen for the season.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="49" t="inlineStr">
+      <c r="A50" s="53" t="inlineStr">
         <is>
           <t>Scoring these results against the model is a holdout look.</t>
         </is>
@@ -21725,124 +21731,124 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="48" t="inlineStr">
+      <c r="A57" s="52" t="inlineStr">
         <is>
           <t>HOW TO USE THIS SHEET</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="49" t="inlineStr"/>
+      <c r="A58" s="53" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="49" t="inlineStr">
+      <c r="A59" s="53" t="inlineStr">
         <is>
           <t>1. Fill the yellow columns only. Everything green is computed.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="49" t="inlineStr"/>
+      <c r="A60" s="53" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="49" t="inlineStr">
+      <c r="A61" s="53" t="inlineStr">
         <is>
           <t>2. 'Settles on' must say what the market actually pays out on. Write 'yellow cards' only if the bookmaker settles on yellows alone. If it says total cards or booking points, BET? shows UNITS? and gives no verdict -- on purpose.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="49" t="inlineStr"/>
+      <c r="A62" s="53" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="49" t="inlineStr">
+      <c r="A63" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">   The model predicts yellows. Counting a red as two cards adds about 5-6 percentage points at every line, always upward, which is larger than the 5% edge threshold. Priced against the wrong market the model shows an OVER edge on nearly every game, and that looks identical to finding an edge.</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="49" t="inlineStr"/>
+      <c r="A64" s="53" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" s="49" t="inlineStr">
+      <c r="A65" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">   The market to look for is 'Yellow Cards', as in the Chelsea screenshot -- not 'Cards' and not 'Booking Points'.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="49" t="inlineStr"/>
+      <c r="A66" s="53" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="49" t="inlineStr">
+      <c r="A67" s="53" t="inlineStr">
         <is>
           <t>3. Record BOTH sides of the price. With one side only, the de-vig cannot run and the implied probability is overstated by the whole margin, which invents edge that is not there.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="49" t="inlineStr"/>
+      <c r="A68" s="53" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="49" t="inlineStr">
+      <c r="A69" s="53" t="inlineStr">
         <is>
           <t>4. Record the price when you see it, before kick-off. A price looked up afterwards is not one you could have taken.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="49" t="inlineStr"/>
+      <c r="A70" s="53" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="49" t="inlineStr">
+      <c r="A71" s="53" t="inlineStr">
         <is>
           <t>5. Stake is EUR 100 a bet. Change the column if you want; the P/L follows it.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="49" t="inlineStr"/>
+      <c r="A72" s="53" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="48" t="inlineStr">
+      <c r="A73" s="52" t="inlineStr">
         <is>
           <t>WHAT THIS SHEET IS AND IS NOT</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="49" t="inlineStr"/>
+      <c r="A74" s="53" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="49" t="inlineStr">
+      <c r="A75" s="53" t="inlineStr">
         <is>
           <t>46 fixtures. A sample this size tells you nothing about whether the model beats a bookmaker -- a verdict on profitability needs thousands of bets. Treat a single week as practice for the workflow.</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="49" t="inlineStr"/>
+      <c r="A76" s="53" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="49" t="inlineStr">
+      <c r="A77" s="53" t="inlineStr">
         <is>
           <t>The referee is 48% of the model's value. If the Referee column says 'not known', the EFL has not published appointments yet (they come one to three days ahead) and these are the weaker version of the model. Re-run run_week_sheet.py for the same dates once they are out and every unplayed row updates.</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="49" t="inlineStr"/>
+      <c r="A78" s="53" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="49" t="inlineStr">
+      <c r="A79" s="53" t="inlineStr">
         <is>
           <t>Model fingerprint d30beac40c73a847, frozen for the season.</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="49" t="inlineStr">
+      <c r="A80" s="53" t="inlineStr">
         <is>
           <t>Scoring these results against the model is a holdout look.</t>
         </is>
@@ -24283,124 +24289,124 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="48" t="inlineStr">
+      <c r="A22" s="52" t="inlineStr">
         <is>
           <t>HOW TO USE THIS SHEET</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="49" t="inlineStr"/>
+      <c r="A23" s="53" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="49" t="inlineStr">
+      <c r="A24" s="53" t="inlineStr">
         <is>
           <t>1. Fill the yellow columns only. Everything green is computed.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="49" t="inlineStr"/>
+      <c r="A25" s="53" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="49" t="inlineStr">
+      <c r="A26" s="53" t="inlineStr">
         <is>
           <t>2. 'Settles on' must say what the market actually pays out on. Write 'yellow cards' only if the bookmaker settles on yellows alone. If it says total cards or booking points, BET? shows UNITS? and gives no verdict -- on purpose.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="49" t="inlineStr"/>
+      <c r="A27" s="53" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="49" t="inlineStr">
+      <c r="A28" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">   The model predicts yellows. Counting a red as two cards adds about 5-6 percentage points at every line, always upward, which is larger than the 5% edge threshold. Priced against the wrong market the model shows an OVER edge on nearly every game, and that looks identical to finding an edge.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="49" t="inlineStr"/>
+      <c r="A29" s="53" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="49" t="inlineStr">
+      <c r="A30" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">   The market to look for is 'Yellow Cards', as in the Chelsea screenshot -- not 'Cards' and not 'Booking Points'.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="49" t="inlineStr"/>
+      <c r="A31" s="53" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="49" t="inlineStr">
+      <c r="A32" s="53" t="inlineStr">
         <is>
           <t>3. Record BOTH sides of the price. With one side only, the de-vig cannot run and the implied probability is overstated by the whole margin, which invents edge that is not there.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="49" t="inlineStr"/>
+      <c r="A33" s="53" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="49" t="inlineStr">
+      <c r="A34" s="53" t="inlineStr">
         <is>
           <t>4. Record the price when you see it, before kick-off. A price looked up afterwards is not one you could have taken.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="49" t="inlineStr"/>
+      <c r="A35" s="53" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="49" t="inlineStr">
+      <c r="A36" s="53" t="inlineStr">
         <is>
           <t>5. Stake is EUR 100 a bet. Change the column if you want; the P/L follows it.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="49" t="inlineStr"/>
+      <c r="A37" s="53" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="48" t="inlineStr">
+      <c r="A38" s="52" t="inlineStr">
         <is>
           <t>WHAT THIS SHEET IS AND IS NOT</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="49" t="inlineStr"/>
+      <c r="A39" s="53" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="49" t="inlineStr">
+      <c r="A40" s="53" t="inlineStr">
         <is>
           <t>11 fixtures. A sample this size tells you nothing about whether the model beats a bookmaker -- a verdict on profitability needs thousands of bets. Treat a single week as practice for the workflow.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="49" t="inlineStr"/>
+      <c r="A41" s="53" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="49" t="inlineStr">
+      <c r="A42" s="53" t="inlineStr">
         <is>
           <t>The referee is 48% of the model's value. If the Referee column says 'not known', the EFL has not published appointments yet (they come one to three days ahead) and these are the weaker version of the model. Re-run run_week_sheet.py for the same dates once they are out and every unplayed row updates.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="49" t="inlineStr"/>
+      <c r="A43" s="53" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="49" t="inlineStr">
+      <c r="A44" s="53" t="inlineStr">
         <is>
           <t>Model fingerprint d30beac40c73a847, frozen for the season.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="49" t="inlineStr">
+      <c r="A45" s="53" t="inlineStr">
         <is>
           <t>Scoring these results against the model is a holdout look.</t>
         </is>
@@ -25001,124 +25007,124 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="52" t="inlineStr">
+      <c r="A12" s="54" t="inlineStr">
         <is>
           <t>HOW TO USE THIS SHEET</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="53" t="inlineStr"/>
+      <c r="A13" s="55" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="53" t="inlineStr">
+      <c r="A14" s="55" t="inlineStr">
         <is>
           <t>1. Fill the yellow columns only. Everything green is computed.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="53" t="inlineStr"/>
+      <c r="A15" s="55" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="53" t="inlineStr">
+      <c r="A16" s="55" t="inlineStr">
         <is>
           <t>2. 'Settles on' must say what the market actually pays out on. Write 'yellow cards' only if the bookmaker settles on yellows alone. If it says total cards or booking points, BET? shows UNITS? and gives no verdict -- on purpose.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="53" t="inlineStr"/>
+      <c r="A17" s="55" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="53" t="inlineStr">
+      <c r="A18" s="55" t="inlineStr">
         <is>
           <t xml:space="preserve">   The model predicts yellows. Counting a red as two cards adds about 5-6 percentage points at every line, always upward, which is larger than the 5% edge threshold. Priced against the wrong market the model shows an OVER edge on nearly every game, and that looks identical to finding an edge.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="53" t="inlineStr"/>
+      <c r="A19" s="55" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="53" t="inlineStr">
+      <c r="A20" s="55" t="inlineStr">
         <is>
           <t xml:space="preserve">   The market to look for is 'Yellow Cards', as in the Chelsea screenshot -- not 'Cards' and not 'Booking Points'.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="53" t="inlineStr"/>
+      <c r="A21" s="55" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="53" t="inlineStr">
+      <c r="A22" s="55" t="inlineStr">
         <is>
           <t>3. Record BOTH sides of the price. With one side only, the de-vig cannot run and the implied probability is overstated by the whole margin, which invents edge that is not there.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="53" t="inlineStr"/>
+      <c r="A23" s="55" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="53" t="inlineStr">
+      <c r="A24" s="55" t="inlineStr">
         <is>
           <t>4. Record the price when you see it, before kick-off. A price looked up afterwards is not one you could have taken.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="53" t="inlineStr"/>
+      <c r="A25" s="55" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="53" t="inlineStr">
+      <c r="A26" s="55" t="inlineStr">
         <is>
           <t>5. Stake is EUR 100 a bet. Change the column if you want; the P/L follows it.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="53" t="inlineStr"/>
+      <c r="A27" s="55" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="52" t="inlineStr">
+      <c r="A28" s="54" t="inlineStr">
         <is>
           <t>WHAT THIS SHEET IS AND IS NOT</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="53" t="inlineStr"/>
+      <c r="A29" s="55" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="53" t="inlineStr">
+      <c r="A30" s="55" t="inlineStr">
         <is>
           <t>1 fixtures. A sample this size tells you nothing about whether the model beats a bookmaker -- a verdict on profitability needs thousands of bets. Treat a single week as practice for the workflow.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="53" t="inlineStr"/>
+      <c r="A31" s="55" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="53" t="inlineStr">
+      <c r="A32" s="55" t="inlineStr">
         <is>
           <t>The referee is 48% of the model's value. If the Referee column says 'not known', the EFL has not published appointments yet (they come one to three days ahead) and these are the weaker version of the model. Re-run run_week_sheet.py for the same dates once they are out and every unplayed row updates.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="53" t="inlineStr"/>
+      <c r="A33" s="55" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="53" t="inlineStr">
+      <c r="A34" s="55" t="inlineStr">
         <is>
           <t>Model fingerprint d30beac40c73a847, frozen for the season.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="53" t="inlineStr">
+      <c r="A35" s="55" t="inlineStr">
         <is>
           <t>Scoring these results against the model is a holdout look.</t>
         </is>

</xml_diff>